<commit_message>
feat(matrix): controles de zoom + actualización de datos
Matriz Apertura × Habilidad:
- Botones zoom-out / zoom-in / reset con 3 niveles:
  Completo (0.5-5.5), 2-5, 3-5 (Campeones).
- Permite aislar el cluster central donde se encimaban etiquetas
  del modo "Por dirección".
- ScatterQuadrants acepta xDomain/yDomain opcionales.

Datos:
- Excel actualizado con 8 nuevas respuestas. El roster.csv actual
  no contiene esos correos, por lo que siguen siendo 61 válidos.
  Pendiente: agregar al roster a mcazarez, kpacheco, surista,
  dgalvez, iwalker, khernandez, vferro, fdamas.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/encuesta.xlsx
+++ b/data/encuesta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://atisa1-my.sharepoint.com/personal/oarredondo_atisa_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C6676785-6D6A-4D25-A304-39537C5CF130}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9F0DF188-C898-4EB2-98D8-EA3E87A06DE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="917" uniqueCount="535">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="584">
   <si>
     <t>Id</t>
   </si>
@@ -1690,6 +1690,153 @@
   </si>
   <si>
     <t>Clasificacion de inventario de insumos medicos</t>
+  </si>
+  <si>
+    <t>mcazarez@atisa.com</t>
+  </si>
+  <si>
+    <t>Maria Del Rosario Cazarez Valdez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ninguna </t>
+  </si>
+  <si>
+    <t xml:space="preserve">no </t>
+  </si>
+  <si>
+    <t>No lo utilizó</t>
+  </si>
+  <si>
+    <t>no se</t>
+  </si>
+  <si>
+    <t>No utilizo AI</t>
+  </si>
+  <si>
+    <t>kpacheco@atisa.com</t>
+  </si>
+  <si>
+    <t>Karla Gabriela Pacheco Garcia</t>
+  </si>
+  <si>
+    <t>Soporte en toma de decisiones;Resumen y síntesis de contenido;Creatividad y Estrategia;Comunicación y Redacción;Organización y planificación;Generación/lluvia de ideas</t>
+  </si>
+  <si>
+    <t>Solo he usado la IA como consulta de algunos artículos de la Ley o consulta de si es correcto algún proceso.</t>
+  </si>
+  <si>
+    <t>Dar formato a los auxiliares que se descargan en Enkontrol</t>
+  </si>
+  <si>
+    <t>surista@atisa.com</t>
+  </si>
+  <si>
+    <t>Sergio Alfredo Urista Vazquez</t>
+  </si>
+  <si>
+    <t>Google Gemini;ChatGPT;Microsoft Copilot;Claude;Canva, Gamma</t>
+  </si>
+  <si>
+    <t>Creatividad y Estrategia;Resumen y síntesis de contenido;Automatización de tareas rutinarias;Generación y edición de contenido visual;Comunicación y Redacción;Soporte en toma de decisiones;Generación/lluvia de ideas;Codificación;Análisis Financiero y de Datos;Organización y planificación;Análisis de Riesgos</t>
+  </si>
+  <si>
+    <t>Correos de notificaciones de control vehicular, y seguridad ocupacional, Análaisis de riesgos de entornos y propuestas basados en normatividad.</t>
+  </si>
+  <si>
+    <t>IBM Environmental Intelligence Suite de IBM, Google Flood Forecasting de Google, DesInventar Sendai de la Organización de las Naciones Unidas, GRCTools, Resolver, RiskWatch, MetricStream, Smartvid.io, Buildots, OpenSpace AI, Palantir Foundry de Palantir Technologies, Azure AI y Digital Twins de Microsoft, SAS Risk Management de SAS Institute, Arantec, ChatGPT de OpenAI, Gemini de Google, Claude de Anthropic.</t>
+  </si>
+  <si>
+    <t>Acceso Tecnológico: Limitaciones en el equipo de cómputo o bloqueos de red para acceder a ciertas IAs.;Aprobación de presupuesto y facturación;Seguridad de Información: Incertidumbre sobre el manejo de datos sensibles de Atisa en plataformas externas.</t>
+  </si>
+  <si>
+    <t>Evaluación de Riesgos e Investigación de Accidentes (Análisis de Causa Raíz)</t>
+  </si>
+  <si>
+    <t>dgalvez@atisa.com</t>
+  </si>
+  <si>
+    <t>Denisse Galvez Ruiz</t>
+  </si>
+  <si>
+    <t>Análisis Financiero y de Datos;Comunicación y Redacción;Automatización de tareas rutinarias;Generación/lluvia de ideas</t>
+  </si>
+  <si>
+    <t>para consultar algunas formulas de excel</t>
+  </si>
+  <si>
+    <t>no lo he aplicado directamente a mis actividades diarias</t>
+  </si>
+  <si>
+    <t>puede ayudarme a checar las horas que reporta Mt con las geocercas(descargadas de plataforma Zeek)</t>
+  </si>
+  <si>
+    <t>iwalker@atisa.com</t>
+  </si>
+  <si>
+    <t>Israel Walker Romero</t>
+  </si>
+  <si>
+    <t>Resumen y síntesis de contenido;Codificación;Creatividad y Estrategia</t>
+  </si>
+  <si>
+    <t>Utilice IA (gemini) para resumir un correo electrónico el cual contenia mucha informacion</t>
+  </si>
+  <si>
+    <t>El lograr detectar en base a un numero "logico" que sensores estan funcionando bien que sensores no funcionan bien</t>
+  </si>
+  <si>
+    <t>khernandez@atisa.com</t>
+  </si>
+  <si>
+    <t>Karely Hernandez Altamirano</t>
+  </si>
+  <si>
+    <t>Automatización de tareas rutinarias;Organización y planificación;Creatividad y Estrategia;Comunicación y Redacción;Generación/lluvia de ideas;Traducción</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Utilice la IA para generar comentarios financieros mas estratégicos y con sentido de negocio </t>
+  </si>
+  <si>
+    <t>Seguridad de Información: Incertidumbre sobre el manejo de datos sensibles de Atisa en plataformas externas.</t>
+  </si>
+  <si>
+    <t>revisión de comentarios financieros o análisis financieros</t>
+  </si>
+  <si>
+    <t>vferro@atisa.com</t>
+  </si>
+  <si>
+    <t>Vanessa</t>
+  </si>
+  <si>
+    <t>ChatGPT;Google Gemini;Claude</t>
+  </si>
+  <si>
+    <t>Automatización de tareas rutinarias;Análisis Financiero y de Datos;Organización y planificación</t>
+  </si>
+  <si>
+    <t>Elaboración de presentaciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claude </t>
+  </si>
+  <si>
+    <t>automatización de reportes</t>
+  </si>
+  <si>
+    <t>fdamas@atisa.com</t>
+  </si>
+  <si>
+    <t>Francisco Javier Damas Arreola</t>
+  </si>
+  <si>
+    <t>Comunicación y Redacción;Análisis Financiero y de Datos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solo utilizo la IA para formalizar ciertos informes </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestión de procesos </t>
   </si>
 </sst>
 </file>
@@ -1725,7 +1872,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1740,10 +1887,6 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1811,8 +1954,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:Q76" totalsRowShown="0">
-  <autoFilter ref="A1:Q76" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:Q84" totalsRowShown="0">
+  <autoFilter ref="A1:Q84" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id" dataDxfId="14">
       <extLst>
@@ -1937,7 +2080,7 @@
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{839C7E11-91E4-4DBD-9C5D-0DEA604FA9AC}">
-      <xlmsforms:msForm id="LQJIR4BlCEiWoiyR9dgtpwK0EwuVtrVOnQmEzdWhWrdUQjYzNFg2V0tDS1JDNFo1U01NQVhKUzg3Qi4u" isFormConnected="1" maxResponseId="75" latestEventMarker="75">
+      <xlmsforms:msForm id="LQJIR4BlCEiWoiyR9dgtpwK0EwuVtrVOnQmEzdWhWrdUQjYzNFg2V0tDS1JDNFo1U01NQVhKUzg3Qi4u" isFormConnected="1" maxResponseId="83" latestEventMarker="83">
         <xlmsforms:syncedQuestionId>id</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>startDate</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>submitDate</xlmsforms:syncedQuestionId>
@@ -2258,7 +2401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q76"/>
+  <dimension ref="A1:Q84"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.140625" customWidth="1"/>
@@ -6147,7 +6290,7 @@
       </c>
     </row>
     <row r="74" spans="1:17" ht="121.5">
-      <c r="A74" s="7">
+      <c r="A74">
         <v>73</v>
       </c>
       <c r="B74" s="2">
@@ -6162,13 +6305,13 @@
       <c r="E74" s="1" t="s">
         <v>515</v>
       </c>
-      <c r="F74" s="8">
+      <c r="F74" s="4">
         <v>5</v>
       </c>
       <c r="G74" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="H74" s="8">
+      <c r="H74" s="4">
         <v>5</v>
       </c>
       <c r="I74" s="1" t="s">
@@ -6200,7 +6343,7 @@
       </c>
     </row>
     <row r="75" spans="1:17" ht="121.5">
-      <c r="A75" s="7">
+      <c r="A75">
         <v>74</v>
       </c>
       <c r="B75" s="2">
@@ -6215,13 +6358,13 @@
       <c r="E75" s="1" t="s">
         <v>521</v>
       </c>
-      <c r="F75" s="8">
+      <c r="F75" s="4">
         <v>5</v>
       </c>
       <c r="G75" s="1" t="s">
         <v>522</v>
       </c>
-      <c r="H75" s="8">
+      <c r="H75" s="4">
         <v>5</v>
       </c>
       <c r="I75" s="1" t="s">
@@ -6253,7 +6396,7 @@
       </c>
     </row>
     <row r="76" spans="1:17" ht="30.75">
-      <c r="A76" s="7">
+      <c r="A76">
         <v>75</v>
       </c>
       <c r="B76" s="2">
@@ -6268,13 +6411,13 @@
       <c r="E76" s="1" t="s">
         <v>529</v>
       </c>
-      <c r="F76" s="8">
+      <c r="F76" s="4">
         <v>2</v>
       </c>
       <c r="G76" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="H76" s="8">
+      <c r="H76" s="4">
         <v>2</v>
       </c>
       <c r="I76" s="1" t="s">
@@ -6303,6 +6446,430 @@
       </c>
       <c r="Q76" s="1" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="77" spans="1:17" ht="25.5" customHeight="1">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" s="2">
+        <v>46129.629409722198</v>
+      </c>
+      <c r="C77" s="2">
+        <v>46129.634548611102</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>535</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="F77" s="4">
+        <v>1</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="H77" s="4">
+        <v>1</v>
+      </c>
+      <c r="I77" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="J77" s="6" t="s">
+        <v>539</v>
+      </c>
+      <c r="K77" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="L77" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="M77" s="6" t="s">
+        <v>541</v>
+      </c>
+      <c r="N77" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="O77" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="P77" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q77" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="78" spans="1:17" ht="60.75">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" s="2">
+        <v>46129.628391203703</v>
+      </c>
+      <c r="C78" s="2">
+        <v>46129.635474536997</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="E78" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="F78" s="4">
+        <v>2</v>
+      </c>
+      <c r="G78" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="H78" s="4">
+        <v>2</v>
+      </c>
+      <c r="I78" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="J78" s="6" t="s">
+        <v>545</v>
+      </c>
+      <c r="K78" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="L78" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="M78" s="6" t="s">
+        <v>546</v>
+      </c>
+      <c r="N78" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="O78" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="P78" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q78" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="79" spans="1:17" ht="244.5">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" s="2">
+        <v>46129.631122685198</v>
+      </c>
+      <c r="C79" s="2">
+        <v>46129.635497685202</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="F79" s="4">
+        <v>5</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="H79" s="4">
+        <v>3</v>
+      </c>
+      <c r="I79" s="1" t="s">
+        <v>550</v>
+      </c>
+      <c r="J79" s="6" t="s">
+        <v>551</v>
+      </c>
+      <c r="K79" s="6" t="s">
+        <v>552</v>
+      </c>
+      <c r="L79" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="M79" s="6" t="s">
+        <v>554</v>
+      </c>
+      <c r="N79" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O79" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P79" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q79" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="80" spans="1:17" ht="60.75">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" s="2">
+        <v>46129.628738425898</v>
+      </c>
+      <c r="C80" s="2">
+        <v>46129.637152777803</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>555</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>556</v>
+      </c>
+      <c r="F80" s="4">
+        <v>3</v>
+      </c>
+      <c r="G80" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="H80" s="4">
+        <v>3</v>
+      </c>
+      <c r="I80" s="1" t="s">
+        <v>557</v>
+      </c>
+      <c r="J80" s="6" t="s">
+        <v>558</v>
+      </c>
+      <c r="K80" s="6" t="s">
+        <v>559</v>
+      </c>
+      <c r="L80" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="M80" s="6" t="s">
+        <v>560</v>
+      </c>
+      <c r="N80" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="O80" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P80" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q80" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="81" spans="1:17" ht="60.75">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" s="2">
+        <v>46129.628993055601</v>
+      </c>
+      <c r="C81" s="2">
+        <v>46129.637280092596</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>561</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>562</v>
+      </c>
+      <c r="F81" s="4">
+        <v>3</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H81" s="4">
+        <v>3</v>
+      </c>
+      <c r="I81" s="1" t="s">
+        <v>563</v>
+      </c>
+      <c r="J81" s="6" t="s">
+        <v>564</v>
+      </c>
+      <c r="K81" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="L81" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="M81" s="6" t="s">
+        <v>565</v>
+      </c>
+      <c r="N81" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="O81" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="P81" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q81" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="82" spans="1:17" ht="60.75">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" s="2">
+        <v>46129.634849536997</v>
+      </c>
+      <c r="C82" s="2">
+        <v>46129.64</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>566</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="F82" s="4">
+        <v>3</v>
+      </c>
+      <c r="G82" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="H82" s="4">
+        <v>3</v>
+      </c>
+      <c r="I82" s="1" t="s">
+        <v>568</v>
+      </c>
+      <c r="J82" s="6" t="s">
+        <v>569</v>
+      </c>
+      <c r="K82" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="L82" s="1" t="s">
+        <v>570</v>
+      </c>
+      <c r="M82" s="6" t="s">
+        <v>571</v>
+      </c>
+      <c r="N82" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="O82" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="P82" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q82" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="83" spans="1:17" ht="30.75">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" s="2">
+        <v>46129.635694444398</v>
+      </c>
+      <c r="C83" s="2">
+        <v>46129.644490740699</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>572</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="F83" s="4">
+        <v>3</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="H83" s="4">
+        <v>3</v>
+      </c>
+      <c r="I83" s="1" t="s">
+        <v>575</v>
+      </c>
+      <c r="J83" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="K83" s="6" t="s">
+        <v>577</v>
+      </c>
+      <c r="L83" s="1" t="s">
+        <v>570</v>
+      </c>
+      <c r="M83" s="6" t="s">
+        <v>578</v>
+      </c>
+      <c r="N83" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="O83" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P83" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q83" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="84" spans="1:17" ht="30.75">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" s="2">
+        <v>46129.651759259301</v>
+      </c>
+      <c r="C84" s="2">
+        <v>46129.659988425898</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>579</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>580</v>
+      </c>
+      <c r="F84" s="4">
+        <v>1</v>
+      </c>
+      <c r="G84" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="H84" s="4">
+        <v>3</v>
+      </c>
+      <c r="I84" s="1" t="s">
+        <v>581</v>
+      </c>
+      <c r="J84" s="6" t="s">
+        <v>582</v>
+      </c>
+      <c r="K84" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="L84" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="M84" s="6" t="s">
+        <v>583</v>
+      </c>
+      <c r="N84" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="O84" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="P84" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q84" s="1" t="s">
+        <v>264</v>
       </c>
     </row>
   </sheetData>

</xml_diff>